<commit_message>
Align historical odds identity with the warehouse hist: contract
Use the same uuid5 match IDs as PR #35, fail closed on naive timestamps
and unknown teams, and keep odds corrections append-only.

Co-authored-by: osmith94 <osmith94@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/examples/historical-odds-export.xlsx
+++ b/docs/examples/historical-odds-export.xlsx
@@ -564,17 +564,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>obs:2157554146f6ffc7f354e49d</t>
+          <t>obs:0022b75d519f57aa509484b7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>hist:48f51c608f13538a8b5552f9</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -584,12 +584,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -624,12 +624,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>draw</t>
+          <t>away</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>3.50</t>
+          <t>3.70</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -667,17 +667,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>obs:3352d49946740e7dde423e20</t>
+          <t>obs:08dab7e79c50f84cde8c99d6</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>hist:43da09c4b3a8524d95032f94</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>championship</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -687,17 +687,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>Leeds United</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>Leicester City</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2025-08-16T14:00:00+00:00</t>
+          <t>2025-08-09T14:00:00+00:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -705,19 +705,9 @@
           <t>synthetic</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>synthetic_book</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>synthetic_book</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>both_teams_to_score</t>
+          <t>match_result</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -727,22 +717,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2025-08-16T12:00:00+00:00</t>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>timestamped</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="U3" t="b">
@@ -750,7 +730,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="W3" t="b">
@@ -768,24 +748,24 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>a1aea63edab3ec737500ca1b6ee4c6ad</t>
+          <t>31a83c87fc53b652bb13fbee15fabf44</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>obs:33ba6b1b13649d5e9744882c</t>
+          <t>obs:09eb48126732794944b1c63e</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>match:8b3c01f634e12086367f71f0</t>
+          <t>hist:ac03200476625d8d800fdf08</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>la-liga</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -795,17 +775,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>chelsea</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2025-08-17T15:30:00+00:00</t>
+          <t>2025-10-26T19:00:00+00:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -815,12 +795,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>synthetic_book</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>synthetic_book</t>
+          <t>synthetic_exchange</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -835,25 +810,45 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>draw</t>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>back</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>2.40</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2025-10-26T17:30:00+00:00</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>closing</t>
+          <t>timestamped</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>5000</t>
         </is>
       </c>
       <c r="U4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="W4" t="b">
@@ -871,24 +866,24 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>fe26f81ef15c9e1885b01e0de490dc5d</t>
+          <t>3bbf470d33cb5e8d72a16a76813ea806</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>obs:3868be1084df8deb2c9f1428</t>
+          <t>obs:0bc4f8931a688d53726860cf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>match:6424b0907156e9ef9757aa46</t>
+          <t>hist:48f51c608f13538a8b5552f9</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>la_liga</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -898,17 +893,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>barcelona</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2025-10-26T19:00:00+00:00</t>
+          <t>2025-08-16T14:00:00+00:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -918,12 +913,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>synthetic_exchange</t>
+          <t>synthetic_book</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>synthetic_book</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>match_result</t>
+          <t>both_teams_to_score</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -933,22 +933,17 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>back</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2025-10-26T17:30:00+00:00</t>
+          <t>2025-08-16T12:00:00+00:00</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -956,22 +951,12 @@
           <t>timestamped</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
       <c r="U5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="W5" t="b">
@@ -989,24 +974,24 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>3bbf470d33cb5e8d72a16a76813ea806</t>
+          <t>a1aea63edab3ec737500ca1b6ee4c6ad</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>obs:3a679c628e1ecb6290fe2719</t>
+          <t>obs:10daf5d5858fa00f344afb3d</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>hist:846a2e49173b5705baad59bc</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1016,17 +1001,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>Chelsea</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2025-08-16T14:00:00+00:00</t>
+          <t>2025-08-17T15:30:00+00:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1036,7 +1021,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>synthetic_exchange</t>
+          <t>synthetic_book</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>synthetic_book</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1051,40 +1041,25 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>draw</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>back</t>
+          <t>away</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>3.40</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>2025-08-16T12:00:00+00:00</t>
+          <t>2.80</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>timestamped</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>800</t>
+          <t>closing</t>
         </is>
       </c>
       <c r="U6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="W6" t="b">
@@ -1102,24 +1077,24 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>3bbf470d33cb5e8d72a16a76813ea806</t>
+          <t>fe26f81ef15c9e1885b01e0de490dc5d</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>obs:3df9be82bd72a5b8833adfd9</t>
+          <t>obs:1561425e8bbdb261d027c3b2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>match:82fd579acbd43b73e02f2fc6</t>
+          <t>hist:ac03200476625d8d800fdf08</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>championship</t>
+          <t>la-liga</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1129,17 +1104,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>leeds united</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>leicester city</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2025-08-09T14:00:00+00:00</t>
+          <t>2025-10-26T19:00:00+00:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1147,6 +1122,11 @@
           <t>synthetic</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>synthetic_exchange</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>match_result</t>
@@ -1159,20 +1139,45 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>unavailable</t>
+          <t>draw</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>3.60</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2025-10-26T17:30:00+00:00</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>timestamped</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>2100</t>
         </is>
       </c>
       <c r="U7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="W7" t="b">
@@ -1190,24 +1195,24 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>31a83c87fc53b652bb13fbee15fabf44</t>
+          <t>3bbf470d33cb5e8d72a16a76813ea806</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>obs:46c39fd3a4cee90f62ee4bd9</t>
+          <t>obs:182a535c6ad25ef7ae17653e</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>hist:48f51c608f13538a8b5552f9</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1217,12 +1222,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1237,17 +1242,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>synthetic_book</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>synthetic_book</t>
+          <t>synthetic_exchange</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>total_goals</t>
+          <t>match_result</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1255,19 +1255,19 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>over</t>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>back</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>1.90</t>
+          <t>3.80</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1280,12 +1280,17 @@
           <t>timestamped</t>
         </is>
       </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
       <c r="U8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="W8" t="b">
@@ -1293,7 +1298,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>regulation_time|full_time|2.5|False|False|False||</t>
+          <t>regulation_time|full_time||False|False|False||</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
@@ -1303,24 +1308,24 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>a1aea63edab3ec737500ca1b6ee4c6ad</t>
+          <t>3bbf470d33cb5e8d72a16a76813ea806</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>obs:6cb12bf0663be39ab68289d6</t>
+          <t>obs:25a1e570476655d0b851d27b</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>hist:48f51c608f13538a8b5552f9</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1330,12 +1335,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1350,17 +1355,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>synthetic_book</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>synthetic_book</t>
+          <t>synthetic_exchange</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>total_goals</t>
+          <t>match_result</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1368,19 +1368,19 @@
           <t>full_time</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>under</t>
+          <t>draw</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>back</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>1.95</t>
+          <t>3.40</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1393,12 +1393,17 @@
           <t>timestamped</t>
         </is>
       </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>800</t>
+        </is>
+      </c>
       <c r="U9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="W9" t="b">
@@ -1406,7 +1411,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>regulation_time|full_time|2.5|False|False|False||</t>
+          <t>regulation_time|full_time||False|False|False||</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
@@ -1416,24 +1421,24 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>a1aea63edab3ec737500ca1b6ee4c6ad</t>
+          <t>3bbf470d33cb5e8d72a16a76813ea806</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>obs:8434477cefca564bae0450c8</t>
+          <t>obs:2742ddfbaf67ca3a888b23ea</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>hist:48f51c608f13538a8b5552f9</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1443,12 +1448,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1473,7 +1478,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>both_teams_to_score</t>
+          <t>total_goals</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1481,14 +1486,19 @@
           <t>full_time</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>over</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>1.90</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1514,7 +1524,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>regulation_time|full_time||False|False|False||</t>
+          <t>regulation_time|full_time|2.5|False|False|False||</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
@@ -1531,17 +1541,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>obs:93b960de5ac37cb68bdf2705</t>
+          <t>obs:304079a78f2931dc7557826a</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>hist:846a2e49173b5705baad59bc</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1551,17 +1561,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>Chelsea</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2025-08-16T14:00:00+00:00</t>
+          <t>2025-08-17T15:30:00+00:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1591,12 +1601,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>home</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>3.70</t>
+          <t>2.60</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1634,17 +1644,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>obs:94fff1c1d4e1850633e35819</t>
+          <t>obs:5470507618688a7f5437a1dc</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>match:6424b0907156e9ef9757aa46</t>
+          <t>hist:48f51c608f13538a8b5552f9</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>la_liga</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1654,17 +1664,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>barcelona</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2025-10-26T19:00:00+00:00</t>
+          <t>2025-08-16T14:00:00+00:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1674,12 +1684,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>synthetic_exchange</t>
+          <t>synthetic_book</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>synthetic_book</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>match_result</t>
+          <t>both_teams_to_score</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1689,22 +1704,17 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>back</t>
+          <t>no</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>2.05</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>2025-10-26T17:30:00+00:00</t>
+          <t>2025-08-16T12:00:00+00:00</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1712,22 +1722,12 @@
           <t>timestamped</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>3300</t>
-        </is>
-      </c>
       <c r="U12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="W12" t="b">
@@ -1745,24 +1745,24 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>3bbf470d33cb5e8d72a16a76813ea806</t>
+          <t>a1aea63edab3ec737500ca1b6ee4c6ad</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>obs:b29a6da138e666daaf1a9e7b</t>
+          <t>obs:6c1560cafd862aab76dabe2c</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>match:6424b0907156e9ef9757aa46</t>
+          <t>hist:48f51c608f13538a8b5552f9</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>la_liga</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1772,17 +1772,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>barcelona</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2025-10-26T19:00:00+00:00</t>
+          <t>2025-08-16T14:00:00+00:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1792,7 +1792,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>synthetic_exchange</t>
+          <t>synthetic_book</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>synthetic_book</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1810,42 +1815,22 @@
           <t>draw</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>back</t>
-        </is>
-      </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>3.60</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>2025-10-26T17:30:00+00:00</t>
+          <t>3.50</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>timestamped</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>2100</t>
+          <t>closing</t>
         </is>
       </c>
       <c r="U13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="W13" t="b">
@@ -1863,24 +1848,24 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>3bbf470d33cb5e8d72a16a76813ea806</t>
+          <t>fe26f81ef15c9e1885b01e0de490dc5d</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>obs:c123aec4edab6295685bf6bd</t>
+          <t>obs:9f67191604927b84ecec5fec</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>match:8b3c01f634e12086367f71f0</t>
+          <t>hist:48f51c608f13538a8b5552f9</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1890,17 +1875,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>chelsea</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2025-08-17T15:30:00+00:00</t>
+          <t>2025-08-16T14:00:00+00:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1920,7 +1905,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>match_result</t>
+          <t>total_goals</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1928,19 +1913,29 @@
           <t>full_time</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>under</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>2025-08-16T12:00:00+00:00</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>closing</t>
+          <t>timestamped</t>
         </is>
       </c>
       <c r="U14" t="b">
@@ -1948,7 +1943,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="W14" t="b">
@@ -1956,7 +1951,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>regulation_time|full_time||False|False|False||</t>
+          <t>regulation_time|full_time|2.5|False|False|False||</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -1966,24 +1961,24 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>fe26f81ef15c9e1885b01e0de490dc5d</t>
+          <t>a1aea63edab3ec737500ca1b6ee4c6ad</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>obs:d38c572d6df12721cd48f4d7</t>
+          <t>obs:a08eda43d1bb828de32ac47d</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>hist:846a2e49173b5705baad59bc</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1993,17 +1988,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>Chelsea</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2025-08-16T14:00:00+00:00</t>
+          <t>2025-08-17T15:30:00+00:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2013,7 +2008,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>synthetic_exchange</t>
+          <t>synthetic_book</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>synthetic_book</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2028,40 +2028,25 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>back</t>
+          <t>draw</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>2025-08-16T12:00:00+00:00</t>
+          <t>3.30</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>timestamped</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>1200</t>
+          <t>closing</t>
         </is>
       </c>
       <c r="U15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="W15" t="b">
@@ -2079,24 +2064,24 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>3bbf470d33cb5e8d72a16a76813ea806</t>
+          <t>fe26f81ef15c9e1885b01e0de490dc5d</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>obs:dd54be1ca14ae45a96903fb3</t>
+          <t>obs:b55890aa565f0339363e083d</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>hist:48f51c608f13538a8b5552f9</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2106,12 +2091,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2129,11 +2114,6 @@
           <t>synthetic_book</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>synthetic_book</t>
-        </is>
-      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>match_result</t>
@@ -2151,12 +2131,17 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>2.20</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>2025-08-16T12:00:00+00:00</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>closing</t>
+          <t>timestamped</t>
         </is>
       </c>
       <c r="U16" t="b">
@@ -2164,16 +2149,11 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="W16" t="b">
-        <v>1</v>
-      </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>regulation_time|full_time||False|False|False||</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2182,24 +2162,24 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>fe26f81ef15c9e1885b01e0de490dc5d</t>
+          <t>b31c7ae0e1e7be277a070daf9a2a2de2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>obs:e003b4dc643d42a363e68850</t>
+          <t>obs:bfd9915d9167a44257ed6d03</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>match:8b3c01f634e12086367f71f0</t>
+          <t>hist:48f51c608f13538a8b5552f9</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2209,17 +2189,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>chelsea</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2025-08-17T15:30:00+00:00</t>
+          <t>2025-08-16T14:00:00+00:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2254,7 +2234,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2.60</t>
+          <t>2.05</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2292,17 +2272,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>obs:e5188d6e943fc12f98a3ad09</t>
+          <t>obs:c10a3fb3f61bdf63bc7a437c</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>hist:ac03200476625d8d800fdf08</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>la-liga</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2312,17 +2292,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2025-08-16T14:00:00+00:00</t>
+          <t>2025-10-26T19:00:00+00:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2357,12 +2337,12 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>3.80</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2025-08-16T12:00:00+00:00</t>
+          <t>2025-10-26T17:30:00+00:00</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2370,9 +2350,14 @@
           <t>timestamped</t>
         </is>
       </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>3300</t>
         </is>
       </c>
       <c r="U18" t="b">
@@ -2405,17 +2390,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>obs:f0fd95e002f9ab8e5d0b8fb9</t>
+          <t>obs:f86c19aba37e2f72850a4776</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>hist:48f51c608f13538a8b5552f9</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2425,12 +2410,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2445,7 +2430,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>synthetic_book</t>
+          <t>synthetic_exchange</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2463,9 +2448,14 @@
           <t>home</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.20</t>
+          <t>2.10</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -2478,16 +2468,26 @@
           <t>timestamped</t>
         </is>
       </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
       <c r="U19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="W19" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>regulation_time|full_time||False|False|False||</t>
+        </is>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>b31c7ae0e1e7be277a070daf9a2a2de2</t>
+          <t>3bbf470d33cb5e8d72a16a76813ea806</t>
         </is>
       </c>
     </row>
@@ -2584,7 +2584,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2631,7 +2631,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2678,7 +2678,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2725,7 +2725,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2772,7 +2772,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>premier_league</t>
+          <t>premier-league</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3054,7 +3054,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>la_liga</t>
+          <t>la-liga</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3101,7 +3101,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>la_liga</t>
+          <t>la-liga</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3148,7 +3148,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>la_liga</t>
+          <t>la-liga</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3195,7 +3195,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>la_liga</t>
+          <t>la-liga</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3242,7 +3242,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>la_liga</t>
+          <t>la-liga</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3289,7 +3289,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>champions_league</t>
+          <t>champions-league</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3330,7 +3330,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>champions_league</t>
+          <t>champions-league</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3371,7 +3371,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>champions_league</t>
+          <t>champions-league</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3412,7 +3412,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>champions_league</t>
+          <t>champions-league</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3453,7 +3453,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>champions_league</t>
+          <t>champions-league</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">

</xml_diff>

<commit_message>
Consume PR #35 match:sha256 facts identity
Stop owning a hist:uuid5 facts catalog. Odds now call the #35
sports_hedge.facts match ID contract and keep timestamp rejection,
append-only corrections, and optional Smarkets.

Co-authored-by: osmith94 <osmith94@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/examples/historical-odds-export.xlsx
+++ b/docs/examples/historical-odds-export.xlsx
@@ -569,12 +569,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>hist:48f51c608f13538a8b5552f9</t>
+          <t>match:506f0a99c52e6b061cdb36f6</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -584,12 +584,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>hist:43da09c4b3a8524d95032f94</t>
+          <t>match:82fd579acbd43b73e02f2fc6</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Leeds United</t>
+          <t>leeds united</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Leicester City</t>
+          <t>leicester city</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -760,12 +760,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>hist:ac03200476625d8d800fdf08</t>
+          <t>match:6424b0907156e9ef9757aa46</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>la-liga</t>
+          <t>la_liga</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -775,12 +775,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>barcelona</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -878,12 +878,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>hist:48f51c608f13538a8b5552f9</t>
+          <t>match:506f0a99c52e6b061cdb36f6</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -986,12 +986,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>hist:846a2e49173b5705baad59bc</t>
+          <t>match:8b3c01f634e12086367f71f0</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1001,12 +1001,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Manchester City</t>
+          <t>manchester city</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>hist:ac03200476625d8d800fdf08</t>
+          <t>match:6424b0907156e9ef9757aa46</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>la-liga</t>
+          <t>la_liga</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1104,12 +1104,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>barcelona</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1207,12 +1207,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>hist:48f51c608f13538a8b5552f9</t>
+          <t>match:506f0a99c52e6b061cdb36f6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1222,12 +1222,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1320,12 +1320,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>hist:48f51c608f13538a8b5552f9</t>
+          <t>match:506f0a99c52e6b061cdb36f6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1433,12 +1433,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>hist:48f51c608f13538a8b5552f9</t>
+          <t>match:506f0a99c52e6b061cdb36f6</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1448,12 +1448,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1546,12 +1546,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>hist:846a2e49173b5705baad59bc</t>
+          <t>match:8b3c01f634e12086367f71f0</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1561,12 +1561,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Manchester City</t>
+          <t>manchester city</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1649,12 +1649,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>hist:48f51c608f13538a8b5552f9</t>
+          <t>match:506f0a99c52e6b061cdb36f6</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1664,12 +1664,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1757,12 +1757,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>hist:48f51c608f13538a8b5552f9</t>
+          <t>match:506f0a99c52e6b061cdb36f6</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1772,12 +1772,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1860,12 +1860,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>hist:48f51c608f13538a8b5552f9</t>
+          <t>match:506f0a99c52e6b061cdb36f6</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1875,12 +1875,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1973,12 +1973,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>hist:846a2e49173b5705baad59bc</t>
+          <t>match:8b3c01f634e12086367f71f0</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1988,12 +1988,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Manchester City</t>
+          <t>manchester city</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2076,12 +2076,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>hist:48f51c608f13538a8b5552f9</t>
+          <t>match:506f0a99c52e6b061cdb36f6</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2091,12 +2091,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>hist:48f51c608f13538a8b5552f9</t>
+          <t>match:506f0a99c52e6b061cdb36f6</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2189,12 +2189,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2277,12 +2277,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>hist:ac03200476625d8d800fdf08</t>
+          <t>match:6424b0907156e9ef9757aa46</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>la-liga</t>
+          <t>la_liga</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2292,12 +2292,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>barcelona</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2395,12 +2395,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>hist:48f51c608f13538a8b5552f9</t>
+          <t>match:506f0a99c52e6b061cdb36f6</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2410,12 +2410,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2584,7 +2584,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2631,7 +2631,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2678,7 +2678,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2725,7 +2725,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2772,7 +2772,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>premier-league</t>
+          <t>premier_league</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3054,7 +3054,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>la-liga</t>
+          <t>la_liga</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3101,7 +3101,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>la-liga</t>
+          <t>la_liga</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3148,7 +3148,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>la-liga</t>
+          <t>la_liga</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3195,7 +3195,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>la-liga</t>
+          <t>la_liga</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3242,7 +3242,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>la-liga</t>
+          <t>la_liga</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3289,7 +3289,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>champions-league</t>
+          <t>champions_league</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3330,7 +3330,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>champions-league</t>
+          <t>champions_league</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3371,7 +3371,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>champions-league</t>
+          <t>champions_league</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3412,7 +3412,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>champions-league</t>
+          <t>champions_league</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3453,7 +3453,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>champions-league</t>
+          <t>champions_league</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">

</xml_diff>

<commit_message>
Rebase odds onto merged facts and fail-closed team mapping
Consume sports_hedge.facts from main (PR #35). Odds mapping resolves
teams through the historical catalog, joins the published Arsenal–Chelsea
match ID, and keeps timestamped paths plus append-only corrections.

Co-authored-by: osmith94 <osmith94@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/examples/historical-odds-export.xlsx
+++ b/docs/examples/historical-odds-export.xlsx
@@ -569,7 +569,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>match:ba5f6ed16933ba065e251522</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>match:ba5f6ed16933ba065e251522</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>match:8b3c01f634e12086367f71f0</t>
+          <t>match:2f329ddd07de34ffa4e679b6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>leeds united</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>match:ba5f6ed16933ba065e251522</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>match:ba5f6ed16933ba065e251522</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>match:ba5f6ed16933ba065e251522</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>match:8b3c01f634e12086367f71f0</t>
+          <t>match:2f329ddd07de34ffa4e679b6</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>leeds united</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>match:ba5f6ed16933ba065e251522</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>match:ba5f6ed16933ba065e251522</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>match:ba5f6ed16933ba065e251522</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>match:8b3c01f634e12086367f71f0</t>
+          <t>match:2f329ddd07de34ffa4e679b6</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1993,7 +1993,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>leeds united</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>match:ba5f6ed16933ba065e251522</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>match:ba5f6ed16933ba065e251522</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>match:506f0a99c52e6b061cdb36f6</t>
+          <t>match:ba5f6ed16933ba065e251522</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">

</xml_diff>